<commit_message>
Atualizando a planilha de erros do Excel
</commit_message>
<xml_diff>
--- a/Plano ou caso de testes.xlsx
+++ b/Plano ou caso de testes.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\SENAI\Desktop\Escola\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SENAI\Desktop\Escola\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F368BC6A-FA5E-4462-B906-582B63A17C61}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DDBA476-3370-4162-9AC3-F0228879BE6F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{2CF0841F-3B4C-4FFF-BE3F-88FA84161A35}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" activeTab="1" xr2:uid="{2CF0841F-3B4C-4FFF-BE3F-88FA84161A35}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Planilha1 (2)" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="61">
   <si>
     <t>TIPO DE TESTE</t>
   </si>
@@ -112,6 +113,102 @@
   </si>
   <si>
     <t>Testando com um número maior que 10</t>
+  </si>
+  <si>
+    <t>Coluna1</t>
+  </si>
+  <si>
+    <t>calcular_media</t>
+  </si>
+  <si>
+    <t>boletim.calculos</t>
+  </si>
+  <si>
+    <t>Teste com notas inteiras</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>[8,10]</t>
+  </si>
+  <si>
+    <t>9.0</t>
+  </si>
+  <si>
+    <t>Teste com notas inteiras e decimais</t>
+  </si>
+  <si>
+    <t>[2, 7.8]</t>
+  </si>
+  <si>
+    <t>4.9</t>
+  </si>
+  <si>
+    <t>Teste com algumas notas inteiras e uma decimal</t>
+  </si>
+  <si>
+    <t>[2,8,7.8]</t>
+  </si>
+  <si>
+    <t>TypeError: '&gt;' not supported between instances of 'str' and 'int'</t>
+  </si>
+  <si>
+    <t>["nove","cinco"]</t>
+  </si>
+  <si>
+    <t>ValueError: A lista de notas não pode estar vazia.</t>
+  </si>
+  <si>
+    <t>Teste com notas em string</t>
+  </si>
+  <si>
+    <t>Teste com lista vazia</t>
+  </si>
+  <si>
+    <t>Teste com apenas uma nota</t>
+  </si>
+  <si>
+    <t>[10]</t>
+  </si>
+  <si>
+    <t>10.0</t>
+  </si>
+  <si>
+    <t>Teste com número negativo</t>
+  </si>
+  <si>
+    <t>[10, -1]</t>
+  </si>
+  <si>
+    <t>4.5</t>
+  </si>
+  <si>
+    <t>TypeError: calcular_media() missing 1 required positional argument: 'notas'</t>
+  </si>
+  <si>
+    <t>()</t>
+  </si>
+  <si>
+    <t>Teste sem lista</t>
+  </si>
+  <si>
+    <t>ValueError: As notas devem ser entre 0 e 10.</t>
+  </si>
+  <si>
+    <t>[20,30]</t>
+  </si>
+  <si>
+    <t>Teste com números maiores que 10</t>
+  </si>
+  <si>
+    <t>Teste com númento inteiro e zero</t>
+  </si>
+  <si>
+    <t>[10, 0]</t>
+  </si>
+  <si>
+    <t>5.0</t>
   </si>
 </sst>
 </file>
@@ -147,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -155,11 +252,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -187,7 +291,7 @@
     <tableColumn id="2" xr3:uid="{8DAF88B1-40DF-432D-8041-39D9653558EB}" name="ARQUIVOS"/>
     <tableColumn id="3" xr3:uid="{00CB3D07-895F-4800-BCDB-C85F097FB672}" name="FUNÇÕES"/>
     <tableColumn id="4" xr3:uid="{A4833CF2-05E3-4AB6-A33F-23FAC96A131A}" name="TESTE"/>
-    <tableColumn id="5" xr3:uid="{D935E0D1-03FD-4DE4-B20E-8CB5B0875399}" name="ENTRADA" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{D935E0D1-03FD-4DE4-B20E-8CB5B0875399}" name="ENTRADA" dataDxfId="3"/>
     <tableColumn id="6" xr3:uid="{B9D78A1A-5733-49DF-9672-38BEE1C6807B}" name="SAÍDA"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -202,8 +306,38 @@
     <tableColumn id="2" xr3:uid="{18EB1B17-CA5F-4A9A-A889-CB005F17C3ED}" name="ARQUIVOS"/>
     <tableColumn id="3" xr3:uid="{49105BF3-6F19-4264-BD8B-5E58A8B644D5}" name="FUNÇÕES"/>
     <tableColumn id="4" xr3:uid="{F433E4DF-CFE6-4D3C-9BED-5B4BD01A5956}" name="TESTE"/>
-    <tableColumn id="5" xr3:uid="{23E42BCA-0E28-46BF-94C1-DDD8849326CF}" name="ENTRADA" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{23E42BCA-0E28-46BF-94C1-DDD8849326CF}" name="ENTRADA" dataDxfId="2"/>
     <tableColumn id="6" xr3:uid="{1D77F3F0-FEC9-4BDE-85C0-585D8B43AC1C}" name="SAÍDA"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{DDAB2C28-02A2-48AC-A935-5ED8BDA42F4C}" name="Tabela15" displayName="Tabela15" ref="A2:F11" totalsRowShown="0">
+  <autoFilter ref="A2:F11" xr:uid="{AD4DC70B-DECB-42B6-850E-CF499EE19F6D}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{63A57E0C-5B1C-4A26-92B8-3D622FCA5F06}" name="TIPO DE TESTE"/>
+    <tableColumn id="2" xr3:uid="{2E6FB21B-EFD8-44CF-A160-A56214EF7FBD}" name="ARQUIVOS"/>
+    <tableColumn id="3" xr3:uid="{82799C25-5FD4-4B69-AF0F-59A4B9816954}" name="FUNÇÕES"/>
+    <tableColumn id="4" xr3:uid="{B80CB860-8F4C-49EA-BA43-BD505D328831}" name="TESTE"/>
+    <tableColumn id="5" xr3:uid="{8755C7AA-6B67-4C92-AFC8-537AABCD3648}" name="ENTRADA" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{F154509F-78B2-4D18-AAD2-114A4AC546E5}" name="SAÍDA"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F9EA7A58-AE32-4AD5-A80D-CBCCD099FA7A}" name="Tabela36" displayName="Tabela36" ref="A14:F21" totalsRowShown="0">
+  <autoFilter ref="A14:F21" xr:uid="{D12EA8B2-E6EA-4F53-9D69-E97F3888CA4A}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{B7098205-E542-4782-9CE3-243E35F6A416}" name="Coluna1"/>
+    <tableColumn id="2" xr3:uid="{335ECF37-B219-4270-B940-C1FBACDAEA9C}" name="ARQUIVOS"/>
+    <tableColumn id="3" xr3:uid="{09AE1071-E524-4D95-96DE-5556D88DBA5D}" name="FUNÇÕES"/>
+    <tableColumn id="4" xr3:uid="{8E6C5C37-9E0F-4AD7-B2CE-AC17593859CE}" name="TESTE"/>
+    <tableColumn id="5" xr3:uid="{6077D1E7-BF57-4435-9B13-C1FB8B18F7EE}" name="ENTRADA" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{E90A61F6-8314-43E3-8D70-4D19C6CEDCD5}" name="SAÍDA"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -808,4 +942,309 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50B9467B-953C-4EE9-BF75-194C170E7125}">
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" customWidth="1"/>
+    <col min="4" max="4" width="58" customWidth="1"/>
+    <col min="5" max="5" width="25.140625" customWidth="1"/>
+    <col min="6" max="6" width="72.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="3">
+        <v>5933333334</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E11" s="1"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>2</v>
+      </c>
+      <c r="D14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" t="s">
+        <v>4</v>
+      </c>
+      <c r="F14" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" t="s">
+        <v>30</v>
+      </c>
+      <c r="D18" t="s">
+        <v>57</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E21" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A13:F13"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="2">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>